<commit_message>
Replace competency question set with canonical Core Leadership Capabilities
Replaces the old 9-question set (Make it Happen / Never Settle /
Choose Right / Smart with Heart) with the canonical 10-question set
across all files:

- src/form-template.html: update SECTIONS array (2 sections, both
  pillar 'Core Leadership Capabilities', 5 competencies each)
- power_automate_payload_reference.json: new payload keys
- 360_feedback_dashboard.xlsx: rebuild FeedbackResponses table with
  new column headers (A2:O8, 15 columns)
- README.md: update Power Automate column mapping table
- SKILL.md: replace canonical question set tables and payload schema

Strengths and Development Areas are unchanged.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/360_feedback_dashboard.xlsx
+++ b/360_feedback_dashboard.xlsx
@@ -178,23 +178,24 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FeedbackResponses" displayName="FeedbackResponses" ref="A2:N8" headerRowCount="1">
-  <autoFilter ref="A2:N8"/>
-  <tableColumns count="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FeedbackResponses" displayName="FeedbackResponses" ref="A2:O8" headerRowCount="1">
+  <autoFilter ref="A2:O8"/>
+  <tableColumns count="15">
     <tableColumn id="1" name="Timestamp"/>
     <tableColumn id="2" name="Subject Name"/>
     <tableColumn id="3" name="Form ID"/>
-    <tableColumn id="4" name="Future Focused"/>
-    <tableColumn id="5" name="Adaptability"/>
-    <tableColumn id="6" name="Positive Outlook"/>
-    <tableColumn id="7" name="Communication"/>
-    <tableColumn id="8" name="Empathy"/>
-    <tableColumn id="9" name="Teamwork"/>
-    <tableColumn id="10" name="Stakeholder Management"/>
-    <tableColumn id="11" name="Planning &amp; Problem Solving"/>
-    <tableColumn id="12" name="Inspirational Leadership"/>
-    <tableColumn id="13" name="Strengths"/>
-    <tableColumn id="14" name="Development Areas"/>
+    <tableColumn id="4" name="Authentic and ethical leadership"/>
+    <tableColumn id="5" name="Emotional intelligence"/>
+    <tableColumn id="6" name="Inspire and influence"/>
+    <tableColumn id="7" name="Change management"/>
+    <tableColumn id="8" name="Team building and collaboration"/>
+    <tableColumn id="9" name="Future focused, innovative, curious and courageous"/>
+    <tableColumn id="10" name="Decision making and problem solving"/>
+    <tableColumn id="11" name="Growth mindset with high self-awareness"/>
+    <tableColumn id="12" name="Cultural competence"/>
+    <tableColumn id="13" name="Communicates with impact"/>
+    <tableColumn id="14" name="Strengths"/>
+    <tableColumn id="15" name="Development Areas"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -489,23 +490,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:O10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="35" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
     <col width="35" customWidth="1" min="14" max="14"/>
+    <col width="35" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -515,7 +517,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="36" customHeight="1">
+    <row r="2" ht="48" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp</t>
@@ -533,55 +535,60 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Future Focused</t>
+          <t>Authentic and ethical leadership</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Adaptability</t>
+          <t>Emotional intelligence</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Positive Outlook</t>
+          <t>Inspire and influence</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Communication</t>
+          <t>Change management</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Empathy</t>
+          <t>Team building and collaboration</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Teamwork</t>
+          <t>Future focused, innovative, curious and courageous</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Stakeholder Management</t>
+          <t>Decision making and problem solving</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Planning &amp; Problem Solving</t>
+          <t>Growth mindset with high self-awareness</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Inspirational Leadership</t>
+          <t>Cultural competence</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
+          <t>Communicates with impact</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
           <t>Strengths</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>Development Areas</t>
         </is>
@@ -609,29 +616,32 @@
         <v>3</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I3" s="4" t="n">
         <v>4</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L3" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="M3" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>Strong communicator. Follows through.</t>
         </is>
       </c>
-      <c r="N3" s="3" t="inlineStr">
+      <c r="O3" s="3" t="inlineStr">
         <is>
           <t>Could delegate more.</t>
         </is>
@@ -668,20 +678,23 @@
         <v>5</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="M4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>Exceptional leadership presence.</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="O4" s="3" t="inlineStr">
         <is>
           <t>More structured planning docs.</t>
         </is>
@@ -709,29 +722,32 @@
         <v>5</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H5" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I5" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="I5" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="J5" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K5" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="L5" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="L5" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="M5" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="N5" s="3" t="inlineStr">
         <is>
           <t>Keeps spirits high under pressure.</t>
         </is>
       </c>
-      <c r="N5" s="3" t="inlineStr">
+      <c r="O5" s="3" t="inlineStr">
         <is>
           <t>More visibility on strategy.</t>
         </is>
@@ -774,14 +790,17 @@
         <v>5</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="M6" s="3" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="N6" s="3" t="inlineStr">
         <is>
           <t>Deep analytical thinker.</t>
         </is>
       </c>
-      <c r="N6" s="3" t="inlineStr">
+      <c r="O6" s="3" t="inlineStr">
         <is>
           <t>More confidence presenting ideas.</t>
         </is>
@@ -826,12 +845,15 @@
       <c r="L7" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="M7" s="3" t="inlineStr">
+      <c r="M7" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N7" s="3" t="inlineStr">
         <is>
           <t>Excellent stakeholder relationships.</t>
         </is>
       </c>
-      <c r="N7" s="3" t="inlineStr">
+      <c r="O7" s="3" t="inlineStr">
         <is>
           <t>Proactive comms could be stronger.</t>
         </is>
@@ -876,12 +898,15 @@
       <c r="L8" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="M8" s="3" t="inlineStr">
+      <c r="M8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N8" s="3" t="inlineStr">
         <is>
           <t>Empathetic, makes time for the team.</t>
         </is>
       </c>
-      <c r="N8" s="3" t="inlineStr">
+      <c r="O8" s="3" t="inlineStr">
         <is>
           <t>More regular 1:1s.</t>
         </is>

</xml_diff>